<commit_message>
IDOL case update: EVENTS E1/E2 + TRIGGERS + MM_PROFILE (03/08)
- EVENTS: E1 ngay 31/07→02/08, note hai khuon canh tranh; E2 ha cap <2%
- TRIGGERS: dien T1-T4 (redeposit, gLSR-flush, pos_r floor, suppressor)
- MM_PROFILE: van tay BIDWALK-A tu so sach (taker<55%, bid-walk 28/07)
- agent_log: session D1-D5 (B1 verify, B3 phan tich, B4 update, B5 dev task)

PENDING operator: DAILY 03/08 dominance=15%/balance=723M sau 04/08 append;
Gate spot vol 03/08; P3 13vi->58bro txhash.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_IDOL.xlsx
+++ b/docs/case_files/CASE_IDOL.xlsx
@@ -3455,6 +3455,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="29">
       <c r="A3" s="55" t="inlineStr">
         <is>
@@ -3480,7 +3481,7 @@
     <row r="4" ht="15" customHeight="1" s="29">
       <c r="A4" s="33" t="inlineStr">
         <is>
-          <t>~07-27→08-01</t>
+          <t>31/07→02/08</t>
         </is>
       </c>
       <c r="B4" s="33" t="inlineStr">
@@ -3495,7 +3496,7 @@
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
-          <t>PENDING-VERIFY: txhash + ngay chinh xac + dich 58bro + label-check</t>
+          <t>PENDING-VERIFY: txhash + ngay chinh xac tu Nansen. Doc: rut TRONG markup (gia len 0.016→0.024 01-02/08) — hai khuon canh tranh: (1) that float leg-2 (ESPORTS-10% pattern) vs (2) chot chien loi pham on-chain. E1 han cap -&gt; P3: can operator feed dia chi + txhash de phan loai.</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3518,7 @@
       </c>
       <c r="D5" s="33" t="inlineStr">
         <is>
-          <t>PENDING-VERIFY: txhash + ma tran BTW-vs-IDOL (B5 chu ky MARKUP da xac nhan?)</t>
+          <t>[HA CAP] &lt;2% supply — khong dang ke tren on-chain thesis. Giu dong lam vet. PENDING-VERIFY: txhash + phan loai BTW-vs-IDOL (Gate wallet 0x0d0707 co phai cung operator BTW khong?)</t>
         </is>
       </c>
     </row>
@@ -3553,7 +3554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="28" min="1" max="1"/>
@@ -3570,6 +3571,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="29">
       <c r="A3" s="55" t="inlineStr">
         <is>
@@ -3598,32 +3600,112 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="29">
-      <c r="A4" s="33" t="n"/>
-      <c r="B4" s="33" t="n"/>
-      <c r="C4" s="33" t="n"/>
-      <c r="D4" s="33" t="n"/>
-      <c r="E4" s="34" t="n"/>
+      <c r="A4" s="33" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>Redeposit bat ky vi nao trong cum 13</t>
+        </is>
+      </c>
+      <c r="C4" s="33" t="inlineStr">
+        <is>
+          <t>Bat ky vi trong cum 13 ~273M gui lai len san (BscScan detect)</t>
+        </is>
+      </c>
+      <c r="D4" s="33" t="inlineStr">
+        <is>
+          <t>DONG AN XA TUC THOI — tiet lo y dinh muon ban; khong gia han wait</t>
+        </is>
+      </c>
+      <c r="E4" s="34" t="inlineStr">
+        <is>
+          <t>CHUA BAT — watcher 0-credit pending B5</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="29">
-      <c r="A5" s="33" t="n"/>
-      <c r="B5" s="33" t="n"/>
-      <c r="C5" s="33" t="n"/>
-      <c r="D5" s="33" t="n"/>
-      <c r="E5" s="34" t="n"/>
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B5" s="33" t="inlineStr">
+        <is>
+          <t>gLSR flush &lt;=1.1 + funding tai ghin &gt;=3d</t>
+        </is>
+      </c>
+      <c r="C5" s="33" t="inlineStr">
+        <is>
+          <t>glsr &lt;= 1.1 lien tuc &gt;=3 nen VA f_avg &lt;= 5e-5 &gt;=3 nen</t>
+        </is>
+      </c>
+      <c r="D5" s="33" t="inlineStr">
+        <is>
+          <t>Ho so re-staging leg-2 song — theo doi luc luong crowd short nap nhien lieu</t>
+        </is>
+      </c>
+      <c r="E5" s="34" t="inlineStr">
+        <is>
+          <t>THEO DOI — 02/08 glsr=1.1436 (can them 03/08 de confirm trend)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="29">
-      <c r="A6" s="33" t="n"/>
-      <c r="B6" s="33" t="n"/>
-      <c r="C6" s="33" t="n"/>
-      <c r="D6" s="33" t="n"/>
-      <c r="E6" s="34" t="n"/>
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>pos_r floor hau-sap</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>pos_r &gt;= 1.6 tai OI floor = con ghe (dinh luat #9); ga &lt; 1.3 = ghe rong</t>
+        </is>
+      </c>
+      <c r="D6" s="33" t="inlineStr">
+        <is>
+          <t>Con ghe -&gt; re-staging kha thi; Ghe rong -&gt; dong an/tra gia gap</t>
+        </is>
+      </c>
+      <c r="E6" s="34" t="inlineStr">
+        <is>
+          <t>THEO DOI — 02/08 pos_r=1.731 (&gt; 1.6, con ghe); OI=10.48M; cho 03/08</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="29">
-      <c r="A7" s="33" t="n"/>
-      <c r="B7" s="33" t="n"/>
-      <c r="C7" s="33" t="n"/>
-      <c r="D7" s="33" t="n"/>
-      <c r="E7" s="34" t="n"/>
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B7" s="33" t="inlineStr">
+        <is>
+          <t>Suppressor bat ky (L-27 §5)</t>
+        </is>
+      </c>
+      <c r="C7" s="33" t="inlineStr">
+        <is>
+          <t>dist_wall &lt; L-27_thresh HOAC neg_div ben &gt;= 3d HOAC post_climax flag</t>
+        </is>
+      </c>
+      <c r="D7" s="33" t="inlineStr">
+        <is>
+          <t>STAND_ASIDE — khong vao/them bat ke phe nao</t>
+        </is>
+      </c>
+      <c r="E7" s="34" t="inlineStr">
+        <is>
+          <t>CHO SO — cols 23/24 chua co gia tri (formula chua tinh)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -3772,7 +3854,7 @@
       </c>
       <c r="B5" s="33" t="inlineStr">
         <is>
-          <t>PENDING — fn=1 chua co du lieu sach 28-31/07; can serie sach sau ignition</t>
+          <t>Sau markup 01/08 (+50% 1 nen), f_avg 02/08 = 5e-5 (san/pinned). Trong nghia: MM chu dong de gim funding ve san sau markup — crowd khong chase (khong co premium demand); CONSISTENT EVAA khuon (re-staging, khong phai climax). Taker 01/08 = 51.5% (&lt;55%) = bid-walk, khong drive up funding. VAN TAY: pin-post-markup + taker&lt;55% = BIDWALK-A fingerprint.</t>
         </is>
       </c>
     </row>
@@ -3784,7 +3866,7 @@
       </c>
       <c r="B6" s="33" t="inlineStr">
         <is>
-          <t>PENDING — 3 van tay cho chot (bid-walk? bait-probe? staging-that?)</t>
+          <t>01/08: vol_q=175.67M (~10x nen binh quan 28-31/07 ~17M), taker=51.5% (duoi 55% suot ca cu markup) — bid-walk ro rang. OI: 27/07 6.60M → 28/07 10.71M (+62%) → 01/08 9.84M → 02/08 10.48M. pos_r: leo 2.059→2.558 truoc ignition, sap 2.524→1.731 sau markup. Timing: top longs loaded 28-31/07 (pre-ignition), exit 02/08 khi crowd gap vao (OI tang nhung pos_r sap). KHUON NGHI VAN: BIDWALK-A (bid limit trong khi taker bearish/neutral).</t>
         </is>
       </c>
     </row>
@@ -3796,7 +3878,7 @@
       </c>
       <c r="B7" s="33" t="inlineStr">
         <is>
-          <t>PENDING — 07-23 vol spike 167M (8x nen) nghi bait-probe; can vol_persistence T+1 xac nhan</t>
+          <t>23/07 vol spike (167M, 8x nen) - bait-probe NGHI VAN (can taker 23/07). 28/07 OI +62% nhung taker=0.480 (bear) = MM mua limit trong khi retail sell. 01/08 markup: taker 51.5% — crowd KHONG phat hien hoac khong dan vao, MM lam gia don gian. 31/07→02/08 rut on-chain 273M TRONG markup = phuc tap: hoac thang float (giam supply san), hoac chot loi on-chain. gLSR: 1.369→1.038 (28/07, crowd giam short) → leo 1.558 (31/07) → sap 1.144 (02/08, crowd tiep tuc unwind).</t>
         </is>
       </c>
     </row>
@@ -3832,7 +3914,7 @@
       </c>
       <c r="B10" s="34" t="inlineStr">
         <is>
-          <t>PENDING — ma tran BTW-vs-IDOL (Gate wallet 0x0d0707 co lien he BTW khong?)</t>
+          <t>PENDING — ma tran BTW-vs-IDOL: Gate wallet 0x0d0707 co lien he BTW khong? E2 ha cap (&lt;2% supply) nhung van giu vet de check cross-campaign. Can: operator feed txhash va label cho 0x0d0707.</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3926,7 @@
       </c>
       <c r="B11" s="34" t="inlineStr">
         <is>
-          <t>PENDING — theo doi sau khi infra_gate label-check xong</t>
+          <t>MM_ID: unknown-IDOL (nghi BIDWALK-A khuon). Du kien 3 van tay can xac nhan: (1) BIDWALK-A: markup taker&lt;55% DONE (01/08 = 51.5%); (2) Bait-probe: vol spike 23/07, PENDING taker; (3) On-chain staging: 7 vi x20M Sent=0 — DONE (giong BANK). Neu bait-probe confirm: so sanh voi AKE/BANK MM_BOOK. Verdict MM_ID: TAM THOI BIDWALK-A, cho them du lieu.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
IDOL Alpha klines + Nansen label + DAILY vol fill
Discovered: /bapi/defi/v1/public/alpha-trade/klines (public, no auth)
IDOL alpha_id=ALPHA_223. Taker ABSTAIN (broken field).

Key numbers:
- 08-01 markup: Alpha vol $11.655M / 50,987 trades (retail peak)
- W2 PASS: Alpha vol 25/07-02/08 = $15.91M >= L-06 $14.97M
- alpha/perp max 0.366x (08-01) — SACH, no suspect

Nansen (operator query): 0x73d8... = Binance DEX/CEX Trading Bot.
273M source confirmed Binance automation, destinations = High Balance unlabeled.

DAILY updated: c36 alpha_suspect, c42 vol_alpha_usd, c43 n_trades_alpha (30 rows)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_IDOL.xlsx
+++ b/docs/case_files/CASE_IDOL.xlsx
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO32"/>
+  <dimension ref="A1:AQ32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -992,6 +992,16 @@
           <t>mm_note</t>
         </is>
       </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>vol_alpha_usd</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>n_trades_alpha</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="15" t="inlineStr">
@@ -1060,14 +1070,19 @@
       <c r="AB3" t="n">
         <v>223517</v>
       </c>
-      <c r="AJ3" s="18">
-        <f>IF(OR(AB3="",D3="",D3=0),"",AB3/D3)</f>
-        <v/>
+      <c r="AJ3" s="18" t="n">
+        <v>89644</v>
       </c>
       <c r="AN3" t="inlineStr">
         <is>
-          <t>Gate=0.2235M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.2235M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.090M n=1,093</t>
+        </is>
+      </c>
+      <c r="AP3" t="n">
+        <v>89644</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>1093</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
@@ -1144,14 +1159,19 @@
       <c r="AB4" t="n">
         <v>261083</v>
       </c>
-      <c r="AJ4" s="18">
-        <f>IF(OR(AB4="",D4="",D4=0),"",AB4/D4)</f>
-        <v/>
+      <c r="AJ4" s="18" t="n">
+        <v>74307</v>
       </c>
       <c r="AN4" t="inlineStr">
         <is>
-          <t>Gate=0.2611M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.2611M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.074M n=1,019</t>
+        </is>
+      </c>
+      <c r="AP4" t="n">
+        <v>74307</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>1019</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -1225,14 +1245,19 @@
       <c r="AB5" t="n">
         <v>1320492</v>
       </c>
-      <c r="AJ5" s="18">
-        <f>IF(OR(AB5="",D5="",D5=0),"",AB5/D5)</f>
-        <v/>
+      <c r="AJ5" s="18" t="n">
+        <v>256301</v>
       </c>
       <c r="AN5" t="inlineStr">
         <is>
-          <t>Gate=1.3205M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=1.3205M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.256M n=2,191</t>
+        </is>
+      </c>
+      <c r="AP5" t="n">
+        <v>256301</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>2191</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -1314,14 +1339,19 @@
       <c r="AB6" t="n">
         <v>1222066</v>
       </c>
-      <c r="AJ6" s="18">
-        <f>IF(OR(AB6="",D6="",D6=0),"",AB6/D6)</f>
-        <v/>
+      <c r="AJ6" s="18" t="n">
+        <v>2064500</v>
       </c>
       <c r="AN6" t="inlineStr">
         <is>
-          <t>Gate=1.2221M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=1.2221M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$2.065M n=5,385</t>
+        </is>
+      </c>
+      <c r="AP6" t="n">
+        <v>2064500</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>5385</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -1403,14 +1433,19 @@
       <c r="AB7" t="n">
         <v>220426</v>
       </c>
-      <c r="AJ7" s="18">
-        <f>IF(OR(AB7="",D7="",D7=0),"",AB7/D7)</f>
-        <v/>
+      <c r="AJ7" s="18" t="n">
+        <v>3410181</v>
       </c>
       <c r="AN7" t="inlineStr">
         <is>
-          <t>Gate=0.2204M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.2204M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$3.410M n=7,249</t>
+        </is>
+      </c>
+      <c r="AP7" t="n">
+        <v>3410181</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>7249</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
@@ -1495,14 +1530,19 @@
       <c r="AB8" t="n">
         <v>379886</v>
       </c>
-      <c r="AJ8" s="18">
-        <f>IF(OR(AB8="",D8="",D8=0),"",AB8/D8)</f>
-        <v/>
+      <c r="AJ8" s="18" t="n">
+        <v>143695</v>
       </c>
       <c r="AN8" t="inlineStr">
         <is>
-          <t>Gate=0.3799M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.3799M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.144M n=1,414</t>
+        </is>
+      </c>
+      <c r="AP8" t="n">
+        <v>143695</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>1414</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
@@ -1584,14 +1624,19 @@
       <c r="AB9" t="n">
         <v>116210</v>
       </c>
-      <c r="AJ9" s="18">
-        <f>IF(OR(AB9="",D9="",D9=0),"",AB9/D9)</f>
-        <v/>
+      <c r="AJ9" s="18" t="n">
+        <v>15239</v>
       </c>
       <c r="AN9" t="inlineStr">
         <is>
-          <t>Gate=0.1162M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.1162M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.015M n=201</t>
+        </is>
+      </c>
+      <c r="AP9" t="n">
+        <v>15239</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>201</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
@@ -1673,14 +1718,19 @@
       <c r="AB10" t="n">
         <v>121348</v>
       </c>
-      <c r="AJ10" s="18">
-        <f>IF(OR(AB10="",D10="",D10=0),"",AB10/D10)</f>
-        <v/>
+      <c r="AJ10" s="18" t="n">
+        <v>2083</v>
       </c>
       <c r="AN10" s="21" t="inlineStr">
         <is>
-          <t>Gate=0.1213M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.1213M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.002M n=45</t>
+        </is>
+      </c>
+      <c r="AP10" t="n">
+        <v>2083</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
@@ -1766,14 +1816,19 @@
       <c r="AB11" t="n">
         <v>85543</v>
       </c>
-      <c r="AJ11" s="18">
-        <f>IF(OR(AB11="",D11="",D11=0),"",AB11/D11)</f>
-        <v/>
+      <c r="AJ11" s="18" t="n">
+        <v>10180</v>
       </c>
       <c r="AN11" s="21" t="inlineStr">
         <is>
-          <t>Gate=0.0855M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.0855M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.010M n=150</t>
+        </is>
+      </c>
+      <c r="AP11" t="n">
+        <v>10180</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>150</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
@@ -1856,14 +1911,19 @@
       <c r="AB12" t="n">
         <v>137097</v>
       </c>
-      <c r="AJ12" s="18">
-        <f>IF(OR(AB12="",D12="",D12=0),"",AB12/D12)</f>
-        <v/>
+      <c r="AJ12" s="18" t="n">
+        <v>17739</v>
       </c>
       <c r="AN12" t="inlineStr">
         <is>
-          <t>Gate=0.1371M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.1371M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.018M n=225</t>
+        </is>
+      </c>
+      <c r="AP12" t="n">
+        <v>17739</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>225</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
@@ -1946,14 +2006,19 @@
       <c r="AB13" t="n">
         <v>356547</v>
       </c>
-      <c r="AJ13" s="18">
-        <f>IF(OR(AB13="",D13="",D13=0),"",AB13/D13)</f>
-        <v/>
+      <c r="AJ13" s="18" t="n">
+        <v>38235</v>
       </c>
       <c r="AN13" t="inlineStr">
         <is>
-          <t>Gate=0.3565M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.3565M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.038M n=509</t>
+        </is>
+      </c>
+      <c r="AP13" t="n">
+        <v>38235</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>509</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
@@ -2036,14 +2101,19 @@
       <c r="AB14" t="n">
         <v>123180</v>
       </c>
-      <c r="AJ14" s="18">
-        <f>IF(OR(AB14="",D14="",D14=0),"",AB14/D14)</f>
-        <v/>
+      <c r="AJ14" s="18" t="n">
+        <v>48308</v>
       </c>
       <c r="AN14" t="inlineStr">
         <is>
-          <t>Gate=0.1232M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.1232M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.048M n=703</t>
+        </is>
+      </c>
+      <c r="AP14" t="n">
+        <v>48308</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>703</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
@@ -2126,15 +2196,20 @@
       <c r="AB15" t="n">
         <v>333231</v>
       </c>
-      <c r="AJ15" s="18">
-        <f>IF(OR(AB15="",D15="",D15=0),"",AB15/D15)</f>
-        <v/>
+      <c r="AJ15" s="18" t="n">
+        <v>25205</v>
       </c>
       <c r="AL15" s="21" t="n"/>
       <c r="AN15" t="inlineStr">
         <is>
-          <t>Gate=0.3332M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.3332M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.025M n=378</t>
+        </is>
+      </c>
+      <c r="AP15" t="n">
+        <v>25205</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>378</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
@@ -2220,14 +2295,19 @@
       <c r="AB16" t="n">
         <v>78360</v>
       </c>
-      <c r="AJ16" s="18">
-        <f>IF(OR(AB16="",D16="",D16=0),"",AB16/D16)</f>
-        <v/>
+      <c r="AJ16" s="18" t="n">
+        <v>11109</v>
       </c>
       <c r="AN16" t="inlineStr">
         <is>
-          <t>Gate=0.0784M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.0784M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.011M n=152</t>
+        </is>
+      </c>
+      <c r="AP16" t="n">
+        <v>11109</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>152</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
@@ -2310,14 +2390,19 @@
       <c r="AB17" t="n">
         <v>88198</v>
       </c>
-      <c r="AJ17" s="18">
-        <f>IF(OR(AB17="",D17="",D17=0),"",AB17/D17)</f>
-        <v/>
+      <c r="AJ17" s="18" t="n">
+        <v>14836</v>
       </c>
       <c r="AN17" t="inlineStr">
         <is>
-          <t>Gate=0.0882M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.0882M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.015M n=199</t>
+        </is>
+      </c>
+      <c r="AP17" t="n">
+        <v>14836</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>199</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
@@ -2400,14 +2485,19 @@
       <c r="AB18" t="n">
         <v>91266</v>
       </c>
-      <c r="AJ18" s="18">
-        <f>IF(OR(AB18="",D18="",D18=0),"",AB18/D18)</f>
-        <v/>
+      <c r="AJ18" s="18" t="n">
+        <v>1236751</v>
       </c>
       <c r="AN18" t="inlineStr">
         <is>
-          <t>Gate=0.0913M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.0913M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$1.237M n=668</t>
+        </is>
+      </c>
+      <c r="AP18" t="n">
+        <v>1236751</v>
+      </c>
+      <c r="AQ18" t="n">
+        <v>668</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
@@ -2490,14 +2580,19 @@
       <c r="AB19" t="n">
         <v>119616</v>
       </c>
-      <c r="AJ19" s="18">
-        <f>IF(OR(AB19="",D19="",D19=0),"",AB19/D19)</f>
-        <v/>
+      <c r="AJ19" s="18" t="n">
+        <v>69050</v>
       </c>
       <c r="AN19" t="inlineStr">
         <is>
-          <t>Gate=0.1196M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.1196M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.069M n=770</t>
+        </is>
+      </c>
+      <c r="AP19" t="n">
+        <v>69050</v>
+      </c>
+      <c r="AQ19" t="n">
+        <v>770</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
@@ -2579,14 +2674,19 @@
       <c r="AB20" t="n">
         <v>75888</v>
       </c>
-      <c r="AJ20" s="18">
-        <f>IF(OR(AB20="",D20="",D20=0),"",AB20/D20)</f>
-        <v/>
+      <c r="AJ20" s="18" t="n">
+        <v>67415</v>
       </c>
       <c r="AN20" t="inlineStr">
         <is>
-          <t>Gate=0.0759M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.0759M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.067M n=575</t>
+        </is>
+      </c>
+      <c r="AP20" t="n">
+        <v>67415</v>
+      </c>
+      <c r="AQ20" t="n">
+        <v>575</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2668,14 +2768,19 @@
       <c r="AB21" t="n">
         <v>77524</v>
       </c>
-      <c r="AJ21" s="18">
-        <f>IF(OR(AB21="",D21="",D21=0),"",AB21/D21)</f>
-        <v/>
+      <c r="AJ21" s="18" t="n">
+        <v>22634</v>
       </c>
       <c r="AN21" t="inlineStr">
         <is>
-          <t>Gate=0.0775M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.0775M | DEX_BSC(PancakeSwap)=N/A | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.023M n=228</t>
+        </is>
+      </c>
+      <c r="AP21" t="n">
+        <v>22634</v>
+      </c>
+      <c r="AQ21" t="n">
+        <v>228</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
@@ -2757,14 +2862,19 @@
       <c r="AB22" t="n">
         <v>1687010</v>
       </c>
-      <c r="AJ22" s="18">
-        <f>IF(OR(AB22="",D22="",D22=0),"",AB22/D22)</f>
-        <v/>
+      <c r="AJ22" s="18" t="n">
+        <v>0.0423</v>
       </c>
       <c r="AN22" t="inlineStr">
         <is>
-          <t>Gate=0.1552M | DEX_BSC(PancakeSwap)=1.5318M | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.1552M | DEX_BSC(PancakeSwap)=1.5318M | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.065M n=567 suspect=0.042x</t>
+        </is>
+      </c>
+      <c r="AP22" t="n">
+        <v>64824</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>567</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
@@ -2849,14 +2959,19 @@
       <c r="AB23" t="n">
         <v>657484</v>
       </c>
-      <c r="AJ23" s="18">
-        <f>IF(OR(AB23="",D23="",D23=0),"",AB23/D23)</f>
-        <v/>
+      <c r="AJ23" s="18" t="n">
+        <v>0.0468</v>
       </c>
       <c r="AN23" t="inlineStr">
         <is>
-          <t>Gate=0.0942M | DEX_BSC(PancakeSwap)=0.5633M | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.0942M | DEX_BSC(PancakeSwap)=0.5633M | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.026M n=261 suspect=0.047x</t>
+        </is>
+      </c>
+      <c r="AP23" t="n">
+        <v>26360</v>
+      </c>
+      <c r="AQ23" t="n">
+        <v>261</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
@@ -2938,14 +3053,19 @@
       <c r="AB24" t="n">
         <v>482966</v>
       </c>
-      <c r="AJ24" s="18">
-        <f>IF(OR(AB24="",D24="",D24=0),"",AB24/D24)</f>
-        <v/>
+      <c r="AJ24" s="18" t="n">
+        <v>0.0278</v>
       </c>
       <c r="AN24" t="inlineStr">
         <is>
-          <t>Gate=0.0287M | DEX_BSC(PancakeSwap)=0.4543M | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.0287M | DEX_BSC(PancakeSwap)=0.4543M | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.013M n=141 suspect=0.028x</t>
+        </is>
+      </c>
+      <c r="AP24" t="n">
+        <v>12611</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>141</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
@@ -3027,14 +3147,19 @@
       <c r="AB25" t="n">
         <v>21594546</v>
       </c>
-      <c r="AJ25" s="18">
-        <f>IF(OR(AB25="",D25="",D25=0),"",AB25/D25)</f>
-        <v/>
+      <c r="AJ25" s="18" t="n">
+        <v>0.2029</v>
       </c>
       <c r="AN25" t="inlineStr">
         <is>
-          <t>Gate=2.9112M | DEX_BSC(PancakeSwap)=18.6833M | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=2.9112M | DEX_BSC(PancakeSwap)=18.6833M | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$3.792M n=27,245 suspect=0.203x</t>
+        </is>
+      </c>
+      <c r="AP25" t="n">
+        <v>3791767</v>
+      </c>
+      <c r="AQ25" t="n">
+        <v>27245</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
@@ -3116,14 +3241,19 @@
       <c r="AB26" t="n">
         <v>12497899</v>
       </c>
-      <c r="AJ26" s="18">
-        <f>IF(OR(AB26="",D26="",D26=0),"",AB26/D26)</f>
-        <v/>
+      <c r="AJ26" s="18" t="n">
+        <v>0.2928</v>
       </c>
       <c r="AN26" t="inlineStr">
         <is>
-          <t>IDOL: no Binance spot. Gate spot 28/07+ via one-shot probe (api.gateio.ws). taker_spot=ABSTAIN (L-29) | Gate=2.6639M | DEX_BSC(PancakeSwap)=9.8340M | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>IDOL: no Binance spot. Gate spot 28/07+ via one-shot probe (api.gateio.ws). taker_spot=ABSTAIN (L-29) | Gate=2.6639M | DEX_BSC(PancakeSwap)=9.8340M | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$2.880M n=14,835 suspect=0.293x</t>
+        </is>
+      </c>
+      <c r="AP26" t="n">
+        <v>2879862</v>
+      </c>
+      <c r="AQ26" t="n">
+        <v>14835</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
@@ -3198,14 +3328,19 @@
       <c r="AB27" t="n">
         <v>2386498</v>
       </c>
-      <c r="AJ27" s="18">
-        <f>IF(OR(AB27="",D27="",D27=0),"",AB27/D27)</f>
-        <v/>
+      <c r="AJ27" s="18" t="n">
+        <v>0.0774</v>
       </c>
       <c r="AN27" t="inlineStr">
         <is>
-          <t>Gate=0.6159M | DEX_BSC(PancakeSwap)=1.7706M | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.6159M | DEX_BSC(PancakeSwap)=1.7706M | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.137M n=1,463 suspect=0.077x</t>
+        </is>
+      </c>
+      <c r="AP27" t="n">
+        <v>137098</v>
+      </c>
+      <c r="AQ27" t="n">
+        <v>1463</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -3280,14 +3415,19 @@
       <c r="AB28" t="n">
         <v>1325917</v>
       </c>
-      <c r="AJ28" s="18">
-        <f>IF(OR(AB28="",D28="",D28=0),"",AB28/D28)</f>
-        <v/>
+      <c r="AJ28" s="18" t="n">
+        <v>0.0994</v>
       </c>
       <c r="AN28" t="inlineStr">
         <is>
-          <t>Gate=0.1990M | DEX_BSC(PancakeSwap)=1.1269M | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.1990M | DEX_BSC(PancakeSwap)=1.1269M | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.112M n=1,169 suspect=0.099x</t>
+        </is>
+      </c>
+      <c r="AP28" t="n">
+        <v>112067</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>1169</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -3362,15 +3502,20 @@
       <c r="AB29" t="n">
         <v>1377252</v>
       </c>
-      <c r="AJ29" s="18">
-        <f>IF(OR(AB29="",D29="",D29=0),"",AB29/D29)</f>
-        <v/>
+      <c r="AJ29" s="18" t="n">
+        <v>0.0784</v>
       </c>
       <c r="AL29" s="21" t="n"/>
       <c r="AN29" s="21" t="inlineStr">
         <is>
-          <t>Gate=0.3526M | DEX_BSC(PancakeSwap)=1.0247M | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.3526M | DEX_BSC(PancakeSwap)=1.0247M | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.080M n=775 suspect=0.078x</t>
+        </is>
+      </c>
+      <c r="AP29" t="n">
+        <v>80310</v>
+      </c>
+      <c r="AQ29" t="n">
+        <v>775</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -3448,14 +3593,19 @@
       </c>
       <c r="AD30" s="17" t="n"/>
       <c r="AE30" s="17" t="n"/>
-      <c r="AJ30" s="18">
-        <f>IF(OR(AB30="",D30="",D30=0),"",AB30/D30)</f>
-        <v/>
+      <c r="AJ30" s="18" t="n">
+        <v>0.1226</v>
       </c>
       <c r="AN30" t="inlineStr">
         <is>
-          <t>Gate=0.1104M | DEX_BSC(PancakeSwap)=1.4345M | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=0.1104M | DEX_BSC(PancakeSwap)=1.4345M | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.176M n=1,398 suspect=0.123x</t>
+        </is>
+      </c>
+      <c r="AP30" t="n">
+        <v>175843</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>1398</v>
       </c>
     </row>
     <row r="31">
@@ -3538,14 +3688,19 @@
         <v>41408688</v>
       </c>
       <c r="AC31" t="n"/>
-      <c r="AJ31">
-        <f>IF(OR(AB31="",D31="",D31=0),"",AB31/D31)</f>
-        <v/>
+      <c r="AJ31" t="n">
+        <v>0.3661</v>
       </c>
       <c r="AN31" t="inlineStr">
         <is>
-          <t>Gate=9.5776M | DEX_BSC(PancakeSwap)=31.8311M | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=9.5776M | DEX_BSC(PancakeSwap)=31.8311M | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$11.655M n=50,987 suspect=0.366x</t>
+        </is>
+      </c>
+      <c r="AP31" t="n">
+        <v>11654883</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>50987</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
@@ -3631,14 +3786,19 @@
         <v>8866587</v>
       </c>
       <c r="AC32" t="n"/>
-      <c r="AJ32">
-        <f>IF(OR(AB32="",D32="",D32=0),"",AB32/D32)</f>
-        <v/>
+      <c r="AJ32" t="n">
+        <v>0.0849</v>
       </c>
       <c r="AN32" t="inlineStr">
         <is>
-          <t>Gate=1.5475M | DEX_BSC(PancakeSwap)=7.3191M | src=GeckoTerminal one-shot 2026-08-03</t>
-        </is>
+          <t>Gate=1.5475M | DEX_BSC(PancakeSwap)=7.3191M | src=GeckoTerminal one-shot 2026-08-03 | alpha_vol=$0.621M n=2,974 suspect=0.085x</t>
+        </is>
+      </c>
+      <c r="AP32" t="n">
+        <v>621160</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>2974</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
IDOL vong-2 Y1-Y5: EVAA re-staging audit 03-05/08 (post_climax watch)
- CASE_IDOL DAILY: append 3 rows 03-05/08 (freshwatch VPS; 05/08 data_bad=1)
  03/08: px=0.01887 gLSR=1.636; 04/08: px=0.01636 gLSR=1.461; 05/08: 1.236
- CASE_IDOL EVENTS: +3 rows 58bro (roundtrip 27.06M net=0 + 32.44M giu lai)
- EVAA checklist: 2/5 dieu kien thoa (iv px giu nen, v khong co suppressor moi)
  gLSR chua flush (1.236 > 1.1); pos_r chua rebuild; funding pin max 1.67d
  OI vs floor 3.92M: +126% — overhead con rat nang
- Y3 58bro: roundtrip 27.06M = THONG DIEP Loai A; net giu 32.44M pending verify
- Y4: framework cho dia chi smart-money khi operator feed (PENDING)
- Y5: CHUA CO GI ro rang; ngay exit SUPPRESSED som nhat: 18/08 (4 dieu kien)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_IDOL.xlsx
+++ b/docs/case_files/CASE_IDOL.xlsx
@@ -75,7 +75,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -130,6 +130,11 @@
         <bgColor rgb="FF375623"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -158,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -210,6 +215,23 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -720,7 +742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ32"/>
+  <dimension ref="A1:AQ35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1016,7 +1038,7 @@
         <v>16584068.48426</v>
       </c>
       <c r="E3" s="18" t="n">
-        <v>0.4780007889437288</v>
+        <v>47.800079</v>
       </c>
       <c r="F3" s="19" t="n">
         <v>5e-05</v>
@@ -1102,7 +1124,7 @@
         <v>16258105.08826</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>0.4760134092685071</v>
+        <v>47.601341</v>
       </c>
       <c r="F4" s="19" t="n">
         <v>5e-05</v>
@@ -1191,7 +1213,7 @@
         <v>15289807.35174</v>
       </c>
       <c r="E5" s="18" t="n">
-        <v>0.4987639777670687</v>
+        <v>49.876398</v>
       </c>
       <c r="F5" s="19" t="n">
         <v>0.000333755</v>
@@ -1277,7 +1299,7 @@
         <v>9154051.07804</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>0.4793609303403439</v>
+        <v>47.936093</v>
       </c>
       <c r="F6" s="19" t="n">
         <v>0.0001978166666666</v>
@@ -1371,7 +1393,7 @@
         <v>8775938.510639999</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>0.4869234392252542</v>
+        <v>48.692344</v>
       </c>
       <c r="F7" s="19" t="n">
         <v>0.0001027616666666</v>
@@ -1465,7 +1487,7 @@
         <v>3998636.20652</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>0.4896940602481673</v>
+        <v>48.969406</v>
       </c>
       <c r="F8" s="19" t="n">
         <v>5e-05</v>
@@ -1562,7 +1584,7 @@
         <v>2234192.34128</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>0.5182033005451896</v>
+        <v>51.82033</v>
       </c>
       <c r="F9" s="19" t="n">
         <v>0.0001081583333333</v>
@@ -1656,7 +1678,7 @@
         <v>2039666.02208</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>0.5287559261604627</v>
+        <v>52.875593</v>
       </c>
       <c r="F10" s="19" t="n">
         <v>7.325333333333333e-05</v>
@@ -1750,7 +1772,7 @@
         <v>1585348.52764</v>
       </c>
       <c r="E11" s="18" t="n">
-        <v>0.4834225092042596</v>
+        <v>48.342251</v>
       </c>
       <c r="F11" s="19" t="n">
         <v>5e-05</v>
@@ -1848,7 +1870,7 @@
         <v>3092893.51746</v>
       </c>
       <c r="E12" s="18" t="n">
-        <v>0.4726014443408847</v>
+        <v>47.260144</v>
       </c>
       <c r="F12" s="19" t="n">
         <v>0.0002229483333333</v>
@@ -1943,7 +1965,7 @@
         <v>5087129.7194</v>
       </c>
       <c r="E13" s="18" t="n">
-        <v>0.4201435632151012</v>
+        <v>42.014356</v>
       </c>
       <c r="F13" s="19" t="n">
         <v>0.00028204</v>
@@ -2038,7 +2060,7 @@
         <v>7737632.26554</v>
       </c>
       <c r="E14" s="18" t="n">
-        <v>0.4939444565350427</v>
+        <v>49.394446</v>
       </c>
       <c r="F14" s="19" t="n">
         <v>0.0001749233333333</v>
@@ -2133,7 +2155,7 @@
         <v>5876711.16144</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>0.4754047375273049</v>
+        <v>47.540474</v>
       </c>
       <c r="F15" s="19" t="n">
         <v>0.00016166</v>
@@ -2229,7 +2251,7 @@
         <v>2231442.34452</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>0.4851628254050874</v>
+        <v>48.516283</v>
       </c>
       <c r="F16" s="19" t="n">
         <v>5e-05</v>
@@ -2327,7 +2349,7 @@
         <v>15102738.57204</v>
       </c>
       <c r="E17" s="18" t="n">
-        <v>0.5092075492693098</v>
+        <v>50.920755</v>
       </c>
       <c r="F17" s="19" t="n">
         <v>0.0001101583333333</v>
@@ -2422,7 +2444,7 @@
         <v>3673663.97688</v>
       </c>
       <c r="E18" s="18" t="n">
-        <v>0.4874717761027368</v>
+        <v>48.747178</v>
       </c>
       <c r="F18" s="19" t="n">
         <v>0.0001210316666666</v>
@@ -2517,7 +2539,7 @@
         <v>24678006.63704</v>
       </c>
       <c r="E19" s="18" t="n">
-        <v>0.4971711271568416</v>
+        <v>49.717113</v>
       </c>
       <c r="F19" s="19" t="n">
         <v>0.0002538166666666</v>
@@ -2612,7 +2634,7 @@
         <v>8491991.76338</v>
       </c>
       <c r="E20" s="18" t="n">
-        <v>0.4962701448405486</v>
+        <v>49.627014</v>
       </c>
       <c r="F20" s="19" t="n">
         <v>0.0001529483333333</v>
@@ -2706,7 +2728,7 @@
         <v>16647813.36078</v>
       </c>
       <c r="E21" s="18" t="n">
-        <v>0.4870963550740638</v>
+        <v>48.709636</v>
       </c>
       <c r="F21" s="19" t="n">
         <v>0.0001377833333333</v>
@@ -2800,7 +2822,7 @@
         <v>7550669.74948</v>
       </c>
       <c r="E22" s="18" t="n">
-        <v>0.4496955742141414</v>
+        <v>44.969557</v>
       </c>
       <c r="F22" s="19" t="n">
         <v>0.0001454166666666</v>
@@ -2894,7 +2916,7 @@
         <v>1919723.54124</v>
       </c>
       <c r="E23" s="18" t="n">
-        <v>0.4756811771186703</v>
+        <v>47.568118</v>
       </c>
       <c r="F23" s="19" t="n">
         <v>5e-05</v>
@@ -2991,7 +3013,7 @@
         <v>1713045.74842</v>
       </c>
       <c r="E24" s="18" t="n">
-        <v>0.5459623019441526</v>
+        <v>54.59623</v>
       </c>
       <c r="F24" s="19" t="n">
         <v>6.360166666666667e-05</v>
@@ -3085,7 +3107,7 @@
         <v>167259563.39932</v>
       </c>
       <c r="E25" s="18" t="n">
-        <v>0.4890935881891488</v>
+        <v>48.909359</v>
       </c>
       <c r="F25" s="19" t="n">
         <v>0.0002468083333333</v>
@@ -3179,7 +3201,7 @@
         <v>16919045.11194</v>
       </c>
       <c r="E26" s="18" t="n">
-        <v>0.4851199670476778</v>
+        <v>48.511997</v>
       </c>
       <c r="F26" s="19" t="n">
         <v>0.0003430716666666</v>
@@ -3273,7 +3295,7 @@
         <v>5930775.03944</v>
       </c>
       <c r="E27" s="18" t="n">
-        <v>0.4801954465121114</v>
+        <v>48.019545</v>
       </c>
       <c r="F27" s="19" t="n">
         <v>0.0001975616666666</v>
@@ -3360,7 +3382,7 @@
         <v>3001087.06951</v>
       </c>
       <c r="E28" s="18" t="n">
-        <v>0.4725181981221648</v>
+        <v>47.25182</v>
       </c>
       <c r="F28" s="19" t="n">
         <v>6.6775e-05</v>
@@ -3447,7 +3469,7 @@
         <v>2995738.46077</v>
       </c>
       <c r="E29" s="18" t="n">
-        <v>0.5284798189362505</v>
+        <v>52.847982</v>
       </c>
       <c r="F29" s="19" t="n">
         <v>9.596166666666668e-05</v>
@@ -3535,7 +3557,7 @@
         <v>7335938.84066</v>
       </c>
       <c r="E30" s="18" t="n">
-        <v>0.4987468671679198</v>
+        <v>49.874687</v>
       </c>
       <c r="F30" s="19" t="n">
         <v>0.00031801</v>
@@ -3625,7 +3647,7 @@
         <v>175671534.50156</v>
       </c>
       <c r="E31" t="n">
-        <v>0.5152925209635985</v>
+        <v>51.529252</v>
       </c>
       <c r="F31" t="n">
         <v>9.492333333333332e-05</v>
@@ -3720,7 +3742,7 @@
         <v>40715280.86713</v>
       </c>
       <c r="E32" t="n">
-        <v>0.500848557452331</v>
+        <v>50.084856</v>
       </c>
       <c r="F32" t="n">
         <v>5e-05</v>
@@ -3800,6 +3822,195 @@
       <c r="AQ32" t="n">
         <v>2974</v>
       </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B33" s="28" t="n">
+        <v>0.018868</v>
+      </c>
+      <c r="C33" s="29" t="n">
+        <v>-0.1838021093656651</v>
+      </c>
+      <c r="D33" s="30" t="n">
+        <v>33874473</v>
+      </c>
+      <c r="E33" t="n">
+        <v>44.555</v>
+      </c>
+      <c r="F33" s="31" t="n">
+        <v>7.166e-05</v>
+      </c>
+      <c r="G33" s="31" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H33" s="31" t="n">
+        <v>0.00017046</v>
+      </c>
+      <c r="I33" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>partial_pin</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="33" t="n">
+        <v>9503666</v>
+      </c>
+      <c r="O33" s="29" t="n">
+        <v>1.8049</v>
+      </c>
+      <c r="P33" s="29" t="n">
+        <v>1.6539</v>
+      </c>
+      <c r="Q33" s="29" t="n">
+        <v>1.6364</v>
+      </c>
+      <c r="R33" s="34" t="n">
+        <v>1.09129935304432</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B34" s="28" t="n">
+        <v>0.016356</v>
+      </c>
+      <c r="C34" s="29" t="n">
+        <v>-0.1331354674581302</v>
+      </c>
+      <c r="D34" s="30" t="n">
+        <v>17027386</v>
+      </c>
+      <c r="E34" t="n">
+        <v>47.177</v>
+      </c>
+      <c r="F34" s="31" t="n">
+        <v>0.0002382</v>
+      </c>
+      <c r="G34" s="31" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H34" s="31" t="n">
+        <v>0.00067558</v>
+      </c>
+      <c r="I34" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>spike</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="33" t="n">
+        <v>8825999</v>
+      </c>
+      <c r="O34" s="29" t="n">
+        <v>1.7453</v>
+      </c>
+      <c r="P34" s="29" t="n">
+        <v>1.6274</v>
+      </c>
+      <c r="Q34" s="29" t="n">
+        <v>1.4612</v>
+      </c>
+      <c r="R34" s="34" t="n">
+        <v>1.07244684773258</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="35" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B35" s="36" t="n">
+        <v>0.01608</v>
+      </c>
+      <c r="C35" s="37" t="n">
+        <v>-0.01687454145267786</v>
+      </c>
+      <c r="D35" s="38" t="n">
+        <v>3100000</v>
+      </c>
+      <c r="E35" s="39" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="F35" s="40" t="n"/>
+      <c r="G35" s="40" t="n"/>
+      <c r="H35" s="40" t="n"/>
+      <c r="I35" s="41" t="n"/>
+      <c r="J35" s="39" t="inlineStr">
+        <is>
+          <t>near_zero</t>
+        </is>
+      </c>
+      <c r="K35" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="42" t="n">
+        <v>8866000</v>
+      </c>
+      <c r="M35" s="39" t="n"/>
+      <c r="N35" s="39" t="n"/>
+      <c r="O35" s="37" t="n">
+        <v>1.841</v>
+      </c>
+      <c r="P35" s="37" t="n">
+        <v>1.322</v>
+      </c>
+      <c r="Q35" s="37" t="n">
+        <v>1.236</v>
+      </c>
+      <c r="R35" s="43" t="n">
+        <v>1.392586989409985</v>
+      </c>
+      <c r="S35" s="39" t="n"/>
+      <c r="T35" s="39" t="n"/>
+      <c r="U35" s="39" t="n"/>
+      <c r="V35" s="39" t="n"/>
+      <c r="W35" s="39" t="n"/>
+      <c r="X35" s="39" t="n"/>
+      <c r="Y35" s="39" t="n"/>
+      <c r="Z35" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA35" s="39" t="n"/>
+      <c r="AB35" s="39" t="n"/>
+      <c r="AC35" s="39" t="n"/>
+      <c r="AD35" s="39" t="n"/>
+      <c r="AE35" s="39" t="n"/>
+      <c r="AF35" s="39" t="n"/>
+      <c r="AG35" s="39" t="n"/>
+      <c r="AH35" s="39" t="n"/>
+      <c r="AI35" s="39" t="n"/>
+      <c r="AJ35" s="39" t="n"/>
+      <c r="AK35" s="39" t="n"/>
+      <c r="AL35" s="39" t="n"/>
+      <c r="AM35" s="39" t="n"/>
+      <c r="AN35" s="39" t="n"/>
+      <c r="AO35" s="39" t="n"/>
+      <c r="AP35" s="39" t="n"/>
+      <c r="AQ35" s="39" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3814,7 +4025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3933,6 +4144,72 @@
       <c r="D9" t="inlineStr">
         <is>
           <t>Suppressor context thường trực: 2%/tháng ngày 11. Markup 01/08 nổ 10 ngày TRƯỚC — unlock ≠ trigger E1 (W6: UNLIKELY). Nguồn: CoinLaunch (op-verified). Team/Strat/Priv vừa ra linear post-cliff 06/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>58bro: nhan 27.06M tokens -&gt; NAP LAI 27.06M cung ngay (roundtrip net=0). Cung ngay nhan them 10M + 14.3M = 24.3M (giu lai, chua nap)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>operator_screenshot_20260806</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>[THONG DIEP?] Gate-&gt;vi-&gt;Gate roundtrip 27.06M = ao cu Loai A; net giu: 24.3M — pending verify co nap tiep khong</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>58bro: nhan 8.14M tokens (giu lai, chua nap theo screenshot)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>operator_screenshot_20260806</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Tong net moi giu (04-06/08): 10M+14.3M+8.14M=32.44M — pending balance check sau 06/08</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Y4 PENDING: dia chi vi smart-money operator thay dang gom — can doi chieu cum 13 vi staging + 58bro + Gate 0x0d0707</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CAN_OPERATOR</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Loai A confirmed: moi on-chain tu he vi cu = THONG DIEP; chi vi ngoai he + swap DEX thuc moi dem</t>
         </is>
       </c>
     </row>

</xml_diff>